<commit_message>
Demo lebih terbatas: tab FULL terkunci dan kapasitas lebih kecil
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ATKdQjtjDkbCW8CD6F26vC
</commit_message>
<xml_diff>
--- a/demo-excel/01-Mini-Akuntansi-demo.xlsx
+++ b/demo-excel/01-Mini-Akuntansi-demo.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NERACA_SALDO" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LABA_RUGI" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NERACA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FULL-DASHBOARD" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="167" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0%;(0.0%);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -112,6 +113,29 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000B1A30"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0033445C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E8449"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -177,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -252,6 +276,12 @@
     </xf>
     <xf numFmtId="167" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="13" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6826,4 +6856,70 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C0392B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="41" t="inlineStr">
+        <is>
+          <t>Fitur Versi Lengkap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="B3" s="42" t="inlineStr">
+        <is>
+          <t>DASHBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>Ringkasan KPI, rasio keuangan, grafik pendapatan vs beban bulanan, dan komposisi beban.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>• Sheet ini hanya tersedia di versi lengkap, lengkap dengan rumus dan grafik yang bekerja dari data Anda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>• Kapasitas data versi lengkap jauh lebih besar dibanding demo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>• Pesan versi lengkap lewat WhatsApp 089623291732.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="B5:C5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>